<commit_message>
QBR: Add date selector
</commit_message>
<xml_diff>
--- a/output/QBR_Workbook.xlsx
+++ b/output/QBR_Workbook.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="155">
   <si>
     <t>KPI</t>
   </si>
@@ -860,10 +860,13 @@
         <v>287</v>
       </c>
       <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
         <v>287</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
       </c>
       <c r="F2">
         <v>287</v>
@@ -877,10 +880,13 @@
         <v>204</v>
       </c>
       <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
         <v>204</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
       </c>
       <c r="F3">
         <v>204</v>
@@ -894,10 +900,13 @@
         <v>10</v>
       </c>
       <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
         <v>10</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
       </c>
       <c r="F4">
         <v>10</v>
@@ -911,10 +920,13 @@
         <v>20</v>
       </c>
       <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
         <v>20</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
       </c>
       <c r="F5">
         <v>20</v>
@@ -928,10 +940,13 @@
         <v>6</v>
       </c>
       <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
         <v>6</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
       </c>
       <c r="F6">
         <v>6</v>
@@ -1155,13 +1170,13 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>287</v>
       </c>
       <c r="C2">
         <v>287</v>
       </c>
       <c r="D2">
-        <v>287</v>
+        <v>0</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1172,13 +1187,13 @@
         <v>7</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>204</v>
       </c>
       <c r="C3">
         <v>204</v>
       </c>
       <c r="D3">
-        <v>204</v>
+        <v>0</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1189,13 +1204,13 @@
         <v>8</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C4">
         <v>10</v>
       </c>
       <c r="D4">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1206,13 +1221,13 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C5">
         <v>20</v>
       </c>
       <c r="D5">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1223,13 +1238,13 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C6">
         <v>6</v>
       </c>
       <c r="D6">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1270,7 +1285,7 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>287</v>
       </c>
       <c r="C2">
         <v>287</v>
@@ -1290,7 +1305,7 @@
         <v>7</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>204</v>
       </c>
       <c r="C3">
         <v>204</v>
@@ -1310,7 +1325,7 @@
         <v>8</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C4">
         <v>10</v>
@@ -1330,7 +1345,7 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C5">
         <v>20</v>
@@ -1350,7 +1365,7 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C6">
         <v>6</v>
@@ -1884,7 +1899,7 @@
         <v>10</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D4">
         <v>10</v>
@@ -1898,7 +1913,7 @@
         <v>20</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D5">
         <v>20</v>
@@ -1912,7 +1927,7 @@
         <v>6</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D6">
         <v>6</v>
@@ -2039,7 +2054,7 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>287</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -2047,7 +2062,7 @@
         <v>7</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -2055,7 +2070,7 @@
         <v>8</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -2063,7 +2078,7 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -2071,17 +2086,23 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
         <v>18</v>
       </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>19</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>